<commit_message>
Join The Council: 🌌🪡 The Starlit Lining Weaver (53)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/RemapDrafts/LumineRemapDraft.xlsx
+++ b/Data/RemapDrafts/LumineRemapDraft.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -456,6 +456,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -467,12 +468,20 @@
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>AlbertGold#2696</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>🌌🪡 The Starlit Lining Weaver: The 53rd member of The Council</t>
         </is>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>